<commit_message>
rebuild exports and reports from the corrected backlog
</commit_message>
<xml_diff>
--- a/sheets/growth_dashboard.xlsx
+++ b/sheets/growth_dashboard.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Scorecard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audience Analysis" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Stability" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mix Adjustment" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel Analysis" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumer Behavior" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Backlog" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality Audit" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Availability" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Campaign Scorecard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Audience Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Segment Stability" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mix Adjustment" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Funnel Analysis" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Consumer Behavior" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Experiment Backlog" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Data Quality Audit" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Metric Availability" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -238,14 +238,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -269,7 +269,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -297,8 +297,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -324,8 +324,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -363,9 +363,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -827,7 +827,7 @@
         <v>0.2123893805309734</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>6.237916694041666</v>
+        <v>6.237916694041665</v>
       </c>
     </row>
     <row r="11">
@@ -1197,12 +1197,12 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="27" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
@@ -1340,10 +1340,10 @@
         <v>2.58120690787931</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>6.237916694041666</v>
+        <v>6.237916694041665</v>
       </c>
       <c r="O2" s="12" t="n">
-        <v>0.0003100067311839313</v>
+        <v>0.0003100067311839312</v>
       </c>
       <c r="P2" s="11" t="n">
         <v>4273.672566371682</v>
@@ -3828,17 +3828,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:AJ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="285" customWidth="1" min="3" max="3"/>
-    <col width="322" customWidth="1" min="4" max="4"/>
+    <col width="479" customWidth="1" min="3" max="3"/>
+    <col width="344" customWidth="1" min="4" max="4"/>
     <col width="88" customWidth="1" min="5" max="5"/>
     <col width="56" customWidth="1" min="6" max="6"/>
     <col width="95" customWidth="1" min="7" max="7"/>
-    <col width="113" customWidth="1" min="8" max="8"/>
+    <col width="148" customWidth="1" min="8" max="8"/>
     <col width="47" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
     <col width="82" customWidth="1" min="11" max="11"/>
@@ -3851,6 +3851,22 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="24" customWidth="1" min="19" max="19"/>
     <col width="103" customWidth="1" min="20" max="20"/>
+    <col width="144" customWidth="1" min="21" max="21"/>
+    <col width="138" customWidth="1" min="22" max="22"/>
+    <col width="51" customWidth="1" min="23" max="23"/>
+    <col width="45" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="47" customWidth="1" min="26" max="26"/>
+    <col width="45" customWidth="1" min="27" max="27"/>
+    <col width="23" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="17" customWidth="1" min="30" max="30"/>
+    <col width="28" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="82" customWidth="1" min="33" max="33"/>
+    <col width="32" customWidth="1" min="34" max="34"/>
+    <col width="142" customWidth="1" min="35" max="35"/>
+    <col width="96" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -3954,6 +3970,86 @@
           <t>PRIORITY REASON</t>
         </is>
       </c>
+      <c r="U1" s="10" t="inlineStr">
+        <is>
+          <t>PROBLEM</t>
+        </is>
+      </c>
+      <c r="V1" s="10" t="inlineStr">
+        <is>
+          <t>OPPORTUNITY</t>
+        </is>
+      </c>
+      <c r="W1" s="10" t="inlineStr">
+        <is>
+          <t>SEGMENT</t>
+        </is>
+      </c>
+      <c r="X1" s="10" t="inlineStr">
+        <is>
+          <t>CHANNEL</t>
+        </is>
+      </c>
+      <c r="Y1" s="10" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="Z1" s="10" t="inlineStr">
+        <is>
+          <t>PRIMARY METRIC</t>
+        </is>
+      </c>
+      <c r="AA1" s="10" t="inlineStr">
+        <is>
+          <t>EXPECTED IMPACT</t>
+        </is>
+      </c>
+      <c r="AB1" s="10" t="inlineStr">
+        <is>
+          <t>MDE</t>
+        </is>
+      </c>
+      <c r="AC1" s="10" t="inlineStr">
+        <is>
+          <t>REQUIRED SAMPLE</t>
+        </is>
+      </c>
+      <c r="AD1" s="10" t="inlineStr">
+        <is>
+          <t>START DATE</t>
+        </is>
+      </c>
+      <c r="AE1" s="10" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="AF1" s="10" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="AG1" s="10" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="AH1" s="10" t="inlineStr">
+        <is>
+          <t>DECISION</t>
+        </is>
+      </c>
+      <c r="AI1" s="10" t="inlineStr">
+        <is>
+          <t>LEARNING</t>
+        </is>
+      </c>
+      <c r="AJ1" s="10" t="inlineStr">
+        <is>
+          <t>NEXT ACTION</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
@@ -3968,12 +4064,12 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>Campaign 1178 scaled budget to $55,662 and achieved lower CPM ($0.27 vs $0.36), but post-click approved conversion collapsed by 73.8% (from 9.22% in Camp 936 to 2.42% in Camp 1178), causing cost per approved conversion to inflate from $15.81 to $63.83.</t>
+          <t>Campaign 1178 spent $55,662.15 (19.2x the budget of Campaign 936 at $2,893.37) and achieved lower CPM ($0.27 vs $0.36), but post-click approved conversion collapsed by 73.8% (from 9.22% in Camp 936 to 2.42% in Camp 1178), causing cost per approved conversion to inflate from $15.81 to $63.83 (+303.7%).</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>Broad-reach ad creatives in Campaign 1178 set generic or misaligned user expectations that fail to convert on the post-click enquiry form. Replacing generic reach hooks with high-intent SMB pain-point hooks (e.g., 'Track daily udhaar payments instantly') will filter low-intent clicks and improve post-click conversion.</t>
+          <t>Broad-reach ad creatives in Campaign 1178 set generic or misaligned user expectations that fail to convert on the post-click enquiry form. Replacing generic reach hooks with high-intent SMB pain-point hooks (e.g., 'Track daily udhaar payments instantly') will filter low-intent clicks and improve downstream conversion without inflating CPA.</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
@@ -4048,6 +4144,84 @@
           <t>Directly attacks the largest source of cost leakage ($48.02 cost-per-approved surge).</t>
         </is>
       </c>
+      <c r="U2" s="14" t="inlineStr">
+        <is>
+          <t>Post-click approved conversion collapsed by 73.8% upon 19.2x budget expansion.</t>
+        </is>
+      </c>
+      <c r="V2" s="14" t="inlineStr">
+        <is>
+          <t>Recover unit cost from $63.83 down towards $28.00 by qualifying click intent upfront.</t>
+        </is>
+      </c>
+      <c r="W2" s="14" t="inlineStr">
+        <is>
+          <t>Scaled Broad Audience (Age 30-49, Top Interests)</t>
+        </is>
+      </c>
+      <c r="X2" s="14" t="inlineStr">
+        <is>
+          <t>Meta Ads (Facebook &amp; Instagram Feed/Reels)</t>
+        </is>
+      </c>
+      <c r="Y2" s="14" t="inlineStr">
+        <is>
+          <t>Growth Marketing Lead</t>
+        </is>
+      </c>
+      <c r="Z2" s="14" t="inlineStr">
+        <is>
+          <t>Click-to-Approved Conversion Rate (%)</t>
+        </is>
+      </c>
+      <c r="AA2" s="14" t="inlineStr">
+        <is>
+          <t>+25% to +35% Lift in Post-Click Conversion</t>
+        </is>
+      </c>
+      <c r="AB2" s="14" t="inlineStr">
+        <is>
+          <t>+25.0% Relative Lift</t>
+        </is>
+      </c>
+      <c r="AC2" s="15" t="n">
+        <v>11369</v>
+      </c>
+      <c r="AD2" s="14" t="inlineStr">
+        <is>
+          <t>Sprint Backlog</t>
+        </is>
+      </c>
+      <c r="AE2" s="14" t="inlineStr">
+        <is>
+          <t>14-day flight upon launch</t>
+        </is>
+      </c>
+      <c r="AF2" s="14" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AG2" s="14" t="inlineStr">
+        <is>
+          <t>Pending execution — target sample size N=11,369 per variant (power 80%, α=0.05)</t>
+        </is>
+      </c>
+      <c r="AH2" s="14" t="inlineStr">
+        <is>
+          <t>Approved for Execution</t>
+        </is>
+      </c>
+      <c r="AI2" s="14" t="inlineStr">
+        <is>
+          <t>Pre-test power analysis demonstrates N=11,369 clicks per variant required to detect a 25% relative lift from the 2.42% baseline.</t>
+        </is>
+      </c>
+      <c r="AJ2" s="14" t="inlineStr">
+        <is>
+          <t>Finalize vernacular creative assets and staging URLs for test launch.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
@@ -4142,6 +4316,84 @@
           <t>High leverage on 36,000+ clicks where 92.6% currently bounce without converting.</t>
         </is>
       </c>
+      <c r="U3" s="14" t="inlineStr">
+        <is>
+          <t>92.6% of clicks bounce on landing page before completing enquiry form.</t>
+        </is>
+      </c>
+      <c r="V3" s="14" t="inlineStr">
+        <is>
+          <t>2-step micro-commitment form reduces cognitive load for Kirana merchants.</t>
+        </is>
+      </c>
+      <c r="W3" s="14" t="inlineStr">
+        <is>
+          <t>All Paid Campaign Post-Click Traffic</t>
+        </is>
+      </c>
+      <c r="X3" s="14" t="inlineStr">
+        <is>
+          <t>Web Landing Page / Mobile Web</t>
+        </is>
+      </c>
+      <c r="Y3" s="14" t="inlineStr">
+        <is>
+          <t>Product Growth Manager (Onboarding)</t>
+        </is>
+      </c>
+      <c r="Z3" s="14" t="inlineStr">
+        <is>
+          <t>Click-to-Total Conversion (Enquiry) Rate (%)</t>
+        </is>
+      </c>
+      <c r="AA3" s="14" t="inlineStr">
+        <is>
+          <t>+20% to +30% Lift in Form Completion</t>
+        </is>
+      </c>
+      <c r="AB3" s="14" t="inlineStr">
+        <is>
+          <t>+20.0% Relative Lift</t>
+        </is>
+      </c>
+      <c r="AC3" s="15" t="n">
+        <v>4250</v>
+      </c>
+      <c r="AD3" s="14" t="inlineStr">
+        <is>
+          <t>Sprint Backlog</t>
+        </is>
+      </c>
+      <c r="AE3" s="14" t="inlineStr">
+        <is>
+          <t>14-day flight upon launch</t>
+        </is>
+      </c>
+      <c r="AF3" s="14" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AG3" s="14" t="inlineStr">
+        <is>
+          <t>Pending execution — target sample size N=4,250 per variant (power 80%, α=0.05)</t>
+        </is>
+      </c>
+      <c r="AH3" s="14" t="inlineStr">
+        <is>
+          <t>Approved for Deployment</t>
+        </is>
+      </c>
+      <c r="AI3" s="14" t="inlineStr">
+        <is>
+          <t>Form analytics instrumentation confirmed as prerequisite; sample size powered for +20% MDE against 7.40% baseline.</t>
+        </is>
+      </c>
+      <c r="AJ3" s="14" t="inlineStr">
+        <is>
+          <t>Instrument step-level telemetry in onboarding form and deploy variant to 50/50 traffic split.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -4156,12 +4408,12 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Segment stability analysis showed that 12 of the 28 interest groups evaluated have &lt; 10 clicks, exhibiting extreme variance in cost per approved conversion, while top interests (e.g. ID 16, 27) demonstrate consistent sub-$25 cost per approved conversion across 50+ click thresholds.</t>
+          <t>Audience segment stability analysis across all 40 interest categories reveals that Interest 27 carries the highest cost per approved conversion at $95.85 (54 conversions on $5,176.17 spend across 3,409 clicks), whereas top efficient scaled interests like ID 16 ($57.34 CPA across 5,144 clicks) and ID 10 ($55.89 CPA across 3,317 clicks) demonstrate proven scale. Reallocating spend away from high-CPA clusters into high-intent stable clusters optimizes blended unit economics.</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Reallocating 30% of media budget away from unstable, fragmented interest segments into the top 5 sample-stable segments will improve overall blended campaign efficiency by eliminating long-tail spend waste.</t>
+          <t>Reallocating 30% of media budget away from inefficient high-CPA interest segments into proven sample-stable segments will improve overall blended campaign efficiency by eliminating long-tail spend waste.</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
@@ -4176,12 +4428,12 @@
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>Fragmented broad targeting across all 30+ interest codes.</t>
+          <t>Fragmented broad targeting across all 40 interest codes.</t>
         </is>
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>Concentrated tier-1 targeting strictly limited to stable interest clusters with &gt;50 clicks history.</t>
+          <t>Concentrated targeting shifting 30% budget from high-CPA interests (e.g. ID 27 at $95.85) to efficient stable interest clusters (IDs 16, 10, 29).</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
@@ -4236,6 +4488,84 @@
           <t>Zero engineering required; actionable immediately within ad campaign budget settings.</t>
         </is>
       </c>
+      <c r="U4" s="14" t="inlineStr">
+        <is>
+          <t>High CPA concentration in interest code 27 ($95.85 CPA) and wide efficiency variance across 40 interest groups.</t>
+        </is>
+      </c>
+      <c r="V4" s="14" t="inlineStr">
+        <is>
+          <t>Reallocate budget from high-CPA segments (e.g., ID 27 at $95.85) to proven efficient segments (e.g., ID 16 at $57.34, ID 10 at $55.89).</t>
+        </is>
+      </c>
+      <c r="W4" s="14" t="inlineStr">
+        <is>
+          <t>Interest Target Groups (Stable vs Volatile)</t>
+        </is>
+      </c>
+      <c r="X4" s="14" t="inlineStr">
+        <is>
+          <t>Meta Ad Account Budget Optimizer</t>
+        </is>
+      </c>
+      <c r="Y4" s="14" t="inlineStr">
+        <is>
+          <t>Performance Marketing Analyst</t>
+        </is>
+      </c>
+      <c r="Z4" s="14" t="inlineStr">
+        <is>
+          <t>Blended Cost per Approved Conversion ($)</t>
+        </is>
+      </c>
+      <c r="AA4" s="14" t="inlineStr">
+        <is>
+          <t>-15% to -22% CPA Reduction</t>
+        </is>
+      </c>
+      <c r="AB4" s="14" t="inlineStr">
+        <is>
+          <t>-15.0% CPA Reduction</t>
+        </is>
+      </c>
+      <c r="AC4" s="15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="AD4" s="14" t="inlineStr">
+        <is>
+          <t>Sprint Backlog</t>
+        </is>
+      </c>
+      <c r="AE4" s="14" t="inlineStr">
+        <is>
+          <t>14-day flight upon launch</t>
+        </is>
+      </c>
+      <c r="AF4" s="14" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AG4" s="14" t="inlineStr">
+        <is>
+          <t>Pending execution — budget reallocation model staged</t>
+        </is>
+      </c>
+      <c r="AH4" s="14" t="inlineStr">
+        <is>
+          <t>Ready for Deployment</t>
+        </is>
+      </c>
+      <c r="AI4" s="14" t="inlineStr">
+        <is>
+          <t>Audit of all 40 interest codes confirmed minimum 128 clicks per segment in the dataset, but CPA ranges from $28 to $95.85.</t>
+        </is>
+      </c>
+      <c r="AJ4" s="14" t="inlineStr">
+        <is>
+          <t>Execute budget shift in campaign settings upon conclusion of current flight.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -4250,12 +4580,12 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>UCI consumer behavior diagnostics show that Returning Visitors have a 3.5x higher purchase rate (16.9% vs 4.8%) and average page value of $7.82 vs $1.15 for New Visitors, but exhibit high exit rates (0.045) on cart pages.</t>
+          <t>UCI consumer diagnostics reveal that Returning Visitors convert at 13.93% (1,470/10,551) compared to 24.91% (422/1,694) for New Visitors—a 44.1% conversion deficit—with an average cart exit rate of 0.0465 and average page value of $5.01 vs $10.77 for New Visitors. Personalizing returning merchant sessions addresses the sharp drop-off observed post-initial visit.</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Displaying a personalized re-engagement banner ('Continue where you left off + free merchant QR setup') to returning visitors within 5 seconds of session start will increase transaction completion.</t>
+          <t>Displaying a personalized re-engagement banner ('Continue where you left off + free merchant QR setup') to returning visitors within 5 seconds of session start will recover returning visitor intent and increase transaction completion.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -4300,7 +4630,7 @@
       </c>
       <c r="M5" s="14" t="inlineStr">
         <is>
-          <t>Quantifies the conversion lift of context-aware personalization for high-intent users.</t>
+          <t>Quantifies the conversion lift of context-aware personalization for returning merchant sessions.</t>
         </is>
       </c>
       <c r="N5" s="14" t="inlineStr">
@@ -4327,7 +4657,85 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>Capitalizes on high baseline intent with proven behavioral divergence.</t>
+          <t>Addresses the 44% conversion degradation in returning visitors who make up 85.6% of sessions.</t>
+        </is>
+      </c>
+      <c r="U5" s="14" t="inlineStr">
+        <is>
+          <t>Returning visitors suffer a 44% lower conversion rate (13.93% vs 24.91% for new visitors) despite representing 85.6% of total sessions.</t>
+        </is>
+      </c>
+      <c r="V5" s="14" t="inlineStr">
+        <is>
+          <t>Contextual 'resume ledger entry' banner to recover returning visitor drop-off.</t>
+        </is>
+      </c>
+      <c r="W5" s="14" t="inlineStr">
+        <is>
+          <t>Returning Visitors (UCI Behavior Diagnostic)</t>
+        </is>
+      </c>
+      <c r="X5" s="14" t="inlineStr">
+        <is>
+          <t>In-App / Mobile Web Banner Nudge</t>
+        </is>
+      </c>
+      <c r="Y5" s="14" t="inlineStr">
+        <is>
+          <t>Lifecycle / CRM Specialist</t>
+        </is>
+      </c>
+      <c r="Z5" s="14" t="inlineStr">
+        <is>
+          <t>Session-to-Purchase Conversion Rate (%)</t>
+        </is>
+      </c>
+      <c r="AA5" s="14" t="inlineStr">
+        <is>
+          <t>+12% to +18% Lift in Return Purchases</t>
+        </is>
+      </c>
+      <c r="AB5" s="14" t="inlineStr">
+        <is>
+          <t>+12.0% Relative Lift</t>
+        </is>
+      </c>
+      <c r="AC5" s="15" t="n">
+        <v>1850</v>
+      </c>
+      <c r="AD5" s="14" t="inlineStr">
+        <is>
+          <t>Sprint Backlog</t>
+        </is>
+      </c>
+      <c r="AE5" s="14" t="inlineStr">
+        <is>
+          <t>14-day flight upon launch</t>
+        </is>
+      </c>
+      <c r="AF5" s="14" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="AG5" s="14" t="inlineStr">
+        <is>
+          <t>Pending execution — backlog scoping</t>
+        </is>
+      </c>
+      <c r="AH5" s="14" t="inlineStr">
+        <is>
+          <t>Approved for Discovery</t>
+        </is>
+      </c>
+      <c r="AI5" s="14" t="inlineStr">
+        <is>
+          <t>UCI dataset shows returning visitors make up 85.6% of sessions (10,551/12,330) but exhibit higher exit rates (0.0465) and lower conversion.</t>
+        </is>
+      </c>
+      <c r="AJ5" s="14" t="inlineStr">
+        <is>
+          <t>Build dynamic cookie-based banner prototype in staging.</t>
         </is>
       </c>
     </row>
@@ -4344,12 +4752,12 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Audience analysis reveals Female segments generate higher CTR (0.024% vs 0.016%) but incur a higher cost per approved conversion ($68.20 vs $42.10 for Males) due to post-click enquiry friction.</t>
+          <t>Audience analysis reveals Female segments generate higher CTR (0.0208% vs 0.0145% for Males, +43.4% higher) but incur higher cost per approved conversion ($69.70 vs $41.44 for Males, +68.2% higher) due to post-click conversion friction (2.07% vs 4.09%).</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Current creative hooks appeal to female SMB owners' visual interest but downstream product copy is tailored predominantly to male-dominated wholesale trade. Creating retail/apparel-specific merchant landing copy for female audiences will bridge the post-click intent gap.</t>
+          <t>Current creative hooks appeal to female SMB owners' visual interest but downstream product copy is tailored predominantly to male-dominated wholesale trade. Creating retail/boutique/apparel-specific merchant landing copy for female audiences will bridge the post-click intent gap.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
@@ -4422,6 +4830,84 @@
       <c r="T6" s="14" t="inlineStr">
         <is>
           <t>High initial click engagement indicates strong top-of-funnel resonance that is currently squandered.</t>
+        </is>
+      </c>
+      <c r="U6" s="14" t="inlineStr">
+        <is>
+          <t>Female segments generate +43.4% higher CTR (0.0208% vs 0.0145%) but 1.68x higher CPA ($69.70 vs $41.44) due to wholesale-biased landing copy.</t>
+        </is>
+      </c>
+      <c r="V6" s="14" t="inlineStr">
+        <is>
+          <t>Verticalized retail/apparel/boutique merchant testimonials and imagery for female cohorts.</t>
+        </is>
+      </c>
+      <c r="W6" s="14" t="inlineStr">
+        <is>
+          <t>Female Business Owners (Age 30-49)</t>
+        </is>
+      </c>
+      <c r="X6" s="14" t="inlineStr">
+        <is>
+          <t>Meta Reels &amp; Vernacular Display</t>
+        </is>
+      </c>
+      <c r="Y6" s="14" t="inlineStr">
+        <is>
+          <t>Creative Strategist / Growth Designer</t>
+        </is>
+      </c>
+      <c r="Z6" s="14" t="inlineStr">
+        <is>
+          <t>Post-Click Approved Conversion Rate (%)</t>
+        </is>
+      </c>
+      <c r="AA6" s="14" t="inlineStr">
+        <is>
+          <t>-20% to -28% CPA for Female Segment</t>
+        </is>
+      </c>
+      <c r="AB6" s="14" t="inlineStr">
+        <is>
+          <t>+20.0% Relative Lift</t>
+        </is>
+      </c>
+      <c r="AC6" s="15" t="n">
+        <v>3100</v>
+      </c>
+      <c r="AD6" s="14" t="inlineStr">
+        <is>
+          <t>Sprint Backlog</t>
+        </is>
+      </c>
+      <c r="AE6" s="14" t="inlineStr">
+        <is>
+          <t>14-day flight upon launch</t>
+        </is>
+      </c>
+      <c r="AF6" s="14" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AG6" s="14" t="inlineStr">
+        <is>
+          <t>Pending execution — creative design backlog</t>
+        </is>
+      </c>
+      <c r="AH6" s="14" t="inlineStr">
+        <is>
+          <t>Ready for Creative Production</t>
+        </is>
+      </c>
+      <c r="AI6" s="14" t="inlineStr">
+        <is>
+          <t>Audience analysis shows Female segments deliver 23,878 clicks / 114.9M impressions (0.0208% CTR) but convert at only 2.07% post-click.</t>
+        </is>
+      </c>
+      <c r="AJ6" s="14" t="inlineStr">
+        <is>
+          <t>Produce 3 vernacular video variants featuring retail store owners.</t>
         </is>
       </c>
     </row>

</xml_diff>